<commit_message>
score not showing bug fix
</commit_message>
<xml_diff>
--- a/UserScore/Gs-1.xlsx
+++ b/UserScore/Gs-1.xlsx
@@ -9501,7 +9501,9 @@
 the Performance of These Schemes</t>
         </is>
       </c>
-      <c r="F403" t="inlineStr"/>
+      <c r="F403" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="n">
@@ -14049,7 +14051,9 @@
           <t xml:space="preserve"> Investment Models </t>
         </is>
       </c>
-      <c r="F606" t="inlineStr"/>
+      <c r="F606" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="607">
       <c r="A607" t="n">

</xml_diff>